<commit_message>
Finishing touches for the architecture of the financial statements section
</commit_message>
<xml_diff>
--- a/backend/fuel-market-information/fuel-market-information.xlsx
+++ b/backend/fuel-market-information/fuel-market-information.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="31.6328125" customWidth="1" min="1" max="1"/>
@@ -1045,102 +1045,6 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>% EBITDA Margin - Aligned</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>OPEX subsidies - Aligned</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Final commit for this proyect
</commit_message>
<xml_diff>
--- a/backend/fuel-market-information/fuel-market-information.xlsx
+++ b/backend/fuel-market-information/fuel-market-information.xlsx
@@ -1,9 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,37 +12,19 @@
     <sheet name="Carbon" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="2">
     <font>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <sz val="8"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -56,42 +39,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -104,22 +57,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -192,7 +139,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -202,44 +149,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -266,32 +213,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -318,24 +247,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -347,162 +258,166 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -516,72 +431,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2030</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2031</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>2032</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>2033</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>2034</t>
         </is>
@@ -794,72 +709,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2030</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2031</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>2032</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>2033</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>2034</t>
         </is>
@@ -1264,72 +1179,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2030</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2031</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>2032</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>2033</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>2034</t>
         </is>

</xml_diff>